<commit_message>
Updated course booking, email notifications, service registration and payment flow
</commit_message>
<xml_diff>
--- a/demo_booking1.xlsx
+++ b/demo_booking1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,6 +496,29 @@
           <t>Friend / Referral</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dhanusha Selvaraj</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dhanusha.selvaraj05@gmail.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>9344520475</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Graduate</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>